<commit_message>
Corregir superficie en PEB completado: 81 m2 a 79.44 m2
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Documentos_Tecnicos/PEB_Pausa_Maule_completado.xlsx
+++ b/03_Documentos_Tecnicos/PEB_Pausa_Maule_completado.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/57b91da64fcc1594/Escritorio/CURSO BIM^MIA/PRACTICO/CLASE 7 SEPTIEMBRE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_F8D0FFC6105FBE3FEC2844B64EA75E7896846D6C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D1EB46AF-7224-4242-8B5D-75933085C50C}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_47CCA5BDD17AFC3FEC2844B64EA69E7ED4F077B4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE55DC64-48BA-4783-8BAC-FE9F638C9B65}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4440" yWindow="4440" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BEP" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
     <t>Superficie</t>
   </si>
   <si>
-    <t>81 m²</t>
+    <t>79.44 m²</t>
   </si>
   <si>
     <t>Plazo</t>
@@ -792,6 +792,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1278,6 +1281,6 @@
     <mergeCell ref="A7:B7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="36" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualizar superficie total en todos los documentos y la web: 79.44 m2 a 79.45 m2 (valor real verificado en Revit)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Documentos_Tecnicos/PEB_Pausa_Maule_completado.xlsx
+++ b/03_Documentos_Tecnicos/PEB_Pausa_Maule_completado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/57b91da64fcc1594/Escritorio/CURSO BIM^MIA/PRACTICO/CLASE 7 SEPTIEMBRE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_47CCA5BDD17AFC3FEC2844B64EA69E7ED4F077B4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE55DC64-48BA-4783-8BAC-FE9F638C9B65}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_858E0603925EBA3FEC2844B64EA69E7EA47AB403" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{638F2765-FBB9-4370-BDD8-FE84BE30EA60}"/>
   <bookViews>
     <workbookView xWindow="4440" yWindow="4440" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55,7 +55,7 @@
     <t>Superficie</t>
   </si>
   <si>
-    <t>79.44 m²</t>
+    <t>79.45 m²</t>
   </si>
   <si>
     <t>Plazo</t>
@@ -277,7 +277,7 @@
     <t>No aplica: Rooms no tienen family type en Revit (TypeId = -1).</t>
   </si>
   <si>
-    <t>Nombre, Numero, Nivel, Area y Perimetro completos en las 9 habitaciones (incluye PASILLO #09, Nivel N1, 2.59 m2, agregada 08-09-2026). Departamento pendiente en las 9. Area total 79.44 m2.</t>
+    <t>Nombre, Numero, Nivel, Area y Perimetro completos en las 9 habitaciones (incluye PASILLO #09, Nivel N1, 2.59 m2, agregada 08-09-2026). Departamento pendiente en las 9. Area total 79.45 m2.</t>
   </si>
   <si>
     <t>Analisis de programa espacial identifica con los primeros campos y contrasta el programa con los siguientes.</t>

</xml_diff>